<commit_message>
Update FIFA World Cup 2026 results data file
</commit_message>
<xml_diff>
--- a/fifa_world_cup_2026_results.xlsx
+++ b/fifa_world_cup_2026_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juan_bohorquez/Documents/repos/world_cup_ampl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEFCECBD-E78D-2148-9745-C3B4AD9F93BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10C542E4-BCA2-F049-BB7A-910E05581693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1040" windowWidth="38400" windowHeight="17440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1300,6 +1300,12 @@
       <c r="A6" t="s">
         <v>6</v>
       </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
       <c r="D6" t="s">
         <v>7</v>
       </c>

</xml_diff>